<commit_message>
fix(metas-gm): atualiza ref com SADA → Edmilson em Q3
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/metas_gm_ref.xlsx
+++ b/backend/metas_gm_ref.xlsx
@@ -3861,17 +3861,17 @@
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -9295,17 +9295,17 @@
       <c r="I65" t="inlineStr"/>
       <c r="J65" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -14679,17 +14679,17 @@
       <c r="I108" t="inlineStr"/>
       <c r="J108" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>DANILO DE SOUZA MACIEIRA</t>
+          <t>Edmilson</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">

</xml_diff>